<commit_message>
Passe a 12 variables : ajoute Sexe/Age/Statut matrimonial/PEPFAR, retire Revenu/Delai
Sexe, Tranche d'age, Statut matrimonial et Soutien PEPFAR deviennent des
variables protegees (conservees quel que soit leur rang statistique, par
analogie avec le cadre OMS 2023 deja applique a l'analyse a 21 variables).
Revenu (redondant avec Depenses mensuelles) et Delai d'attente sont retires
des candidats. Le notebook re-entraine les 4 modeles sur ces 12 variables et
exporte le meilleur (Regression Logistique, F1=0.535) vers l'application.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modeles/performances_modeles.xlsx
+++ b/modeles/performances_modeles.xlsx
@@ -482,28 +482,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6554054054054054</v>
+        <v>0.6418918918918919</v>
       </c>
       <c r="C2" t="n">
         <v>0.7171717171717171</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4641148325358851</v>
+        <v>0.4589371980676328</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5434173669467787</v>
+        <v>0.5352112676056338</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7678303303303304</v>
+        <v>0.7533271908271908</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5569858936052914</v>
+        <v>0.550903673169217</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2006391994774515</v>
+        <v>0.2018577628715015</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5700000000000003</v>
+        <v>0.5600000000000003</v>
       </c>
     </row>
     <row r="3">
@@ -513,28 +513,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6554054054054054</v>
+        <v>0.5540540540540541</v>
       </c>
       <c r="C3" t="n">
         <v>0.7727272727272727</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5187165775401069</v>
+        <v>0.4767441860465116</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5791044776119403</v>
+        <v>0.5125</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7750819000819001</v>
+        <v>0.7440281190281191</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5525657820372009</v>
+        <v>0.5382839795010335</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1995417920456778</v>
+        <v>0.1948166925063578</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5000000000000002</v>
+        <v>0.5200000000000002</v>
       </c>
     </row>
     <row r="4">
@@ -544,28 +544,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2905405405405405</v>
+        <v>0.3243243243243243</v>
       </c>
       <c r="C4" t="n">
         <v>0.9570707070707071</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7166666666666667</v>
+        <v>0.7384615384615385</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4134615384615384</v>
+        <v>0.4507042253521127</v>
       </c>
       <c r="F4" t="n">
-        <v>0.767949767949768</v>
+        <v>0.7534636909636909</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5556836236255458</v>
+        <v>0.5492188981679338</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1615405287270204</v>
+        <v>0.1620685292689652</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3300000000000001</v>
+        <v>0.3200000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -575,28 +575,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.6351351351351351</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7095959595959596</v>
+        <v>0.7146464646464646</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4549763033175355</v>
+        <v>0.4541062801932367</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5348189415041783</v>
+        <v>0.5295774647887324</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7497952497952498</v>
+        <v>0.7309326371826371</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5371852480136197</v>
+        <v>0.5323834932975727</v>
       </c>
       <c r="H5" t="n">
-        <v>0.200491264462471</v>
+        <v>0.2017050385475159</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5500000000000003</v>
+        <v>0.5700000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Passe a 14 variables (Soutien_Familial, Traitement_Alternatif) et selection sur score composite
Le formulaire, le recap, le PDF, le scoring par lot et le diagnostic
ignoraient silencieusement les 2 nouvelles variables demandees par le
CNLS (toujours evaluees a leur categorie de reference). Corrige partout.

Selection du modele deploye : score composite (moyenne a poids egal de
Sensibilite, Specificite, Precision, AUC-ROC, AUC-PR, 1-Brier) au lieu
du seul F1-Score, pour ne sacrifier aucune dimension clinique. Corrige
aussi une incoherence : les metriques de comparaison etaient evaluees a
un seuil fixe de 0.50 au lieu du seuil optimal propre a chaque modele
(le seuil reellement deploye). Random Forest retenu (Rappel 61.5% /
Specificite 80% / Precision 53.5%), plus equilibre que le SVM que le
score composite aurait choisi sur l'ancienne evaluation au seuil fixe.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modeles/performances_modeles.xlsx
+++ b/modeles/performances_modeles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Score composite</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Seuil optimal</t>
         </is>
       </c>
@@ -482,28 +487,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6418918918918919</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7171717171717171</v>
+        <v>0.8434343434343434</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4589371980676328</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5352112676056338</v>
+        <v>0.5314685314685315</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7533271908271908</v>
+        <v>0.7607067294567296</v>
       </c>
       <c r="G2" t="n">
-        <v>0.550903673169217</v>
+        <v>0.5490358841670169</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2018577628715015</v>
+        <v>0.1998676384934421</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5600000000000003</v>
+        <v>0.6695912449598868</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.5800000000000003</v>
       </c>
     </row>
     <row r="3">
@@ -513,28 +521,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5540540540540541</v>
+        <v>0.6148648648648649</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.8005050505050505</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4767441860465116</v>
+        <v>0.5352941176470588</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5125</v>
+        <v>0.5723270440251572</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7440281190281191</v>
+        <v>0.7606726044226044</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5382839795010335</v>
+        <v>0.5474789994265754</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1948166925063578</v>
+        <v>0.1948384128711323</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5200000000000002</v>
+        <v>0.6773295373325036</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.5000000000000002</v>
       </c>
     </row>
     <row r="4">
@@ -544,28 +555,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3243243243243243</v>
+        <v>0.5945945945945946</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9570707070707071</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7384615384615385</v>
+        <v>0.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4507042253521127</v>
+        <v>0.5432098765432098</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7534636909636909</v>
+        <v>0.7626006688506688</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5492188981679338</v>
+        <v>0.550225415019167</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1620685292689652</v>
+        <v>0.1611786563777481</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3200000000000001</v>
+        <v>0.6706699666440766</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.2900000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -575,28 +589,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6283783783783784</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7146464646464646</v>
+        <v>0.7929292929292929</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4541062801932367</v>
+        <v>0.5314285714285715</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5295774647887324</v>
+        <v>0.5758513931888545</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7309326371826371</v>
+        <v>0.751748907998908</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5323834932975727</v>
+        <v>0.5369405983378899</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2017050385475159</v>
+        <v>0.1963230818510056</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5700000000000003</v>
+        <v>0.6741837778703393</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5300000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>